<commit_message>
fixed issues with sports icons
</commit_message>
<xml_diff>
--- a/backend/data/EventData.xlsx
+++ b/backend/data/EventData.xlsx
@@ -426,7 +426,7 @@
         <v>Foosball</v>
       </c>
       <c r="C2" t="str">
-        <v>/icons/foosball.svg</v>
+        <v>/Icons/foosball.svg</v>
       </c>
       <c r="D2" t="str">
         <v>Table soccer played with rods and miniature players, requiring quick reflexes and strategic play.</v>
@@ -440,7 +440,7 @@
         <v>Carrom</v>
       </c>
       <c r="C3" t="str">
-        <v>/icons/carrom.svg</v>
+        <v>/Icons/carrom.svg</v>
       </c>
       <c r="D3" t="str">
         <v>Fast-paced tabletop game where players flick discs into pockets, combining skill and strategy.</v>
@@ -454,7 +454,7 @@
         <v>Chess</v>
       </c>
       <c r="C4" t="str">
-        <v>/icons/chess.svg</v>
+        <v>/Icons/chess.svg</v>
       </c>
       <c r="D4" t="str">
         <v>Classic strategic board game of kings and queens, testing players' tactical thinking.</v>
@@ -468,7 +468,7 @@
         <v>Table Tennis</v>
       </c>
       <c r="C5" t="str">
-        <v>/icons/table-tennis.svg</v>
+        <v>/Icons/table-tennis.svg</v>
       </c>
       <c r="D5" t="str">
         <v>Fast-paced racket sport played on a table, demanding quick reflexes and precision.</v>
@@ -482,7 +482,7 @@
         <v>Badminton</v>
       </c>
       <c r="C6" t="str">
-        <v>/icons/badminton.svg</v>
+        <v>/Icons/badminton.svg</v>
       </c>
       <c r="D6" t="str">
         <v>High-energy racket sport played with a shuttlecock, requiring agility and tactical play.</v>
@@ -496,7 +496,7 @@
         <v>Cricket</v>
       </c>
       <c r="C7" t="str">
-        <v>/icons/cricket.svg</v>
+        <v>/Icons/cricket.svg</v>
       </c>
       <c r="D7" t="str">
         <v>Team sport played with bat and ball, combining individual skill with team strategy.</v>
@@ -510,7 +510,7 @@
         <v>Football</v>
       </c>
       <c r="C8" t="str">
-        <v>/icons/football.svg</v>
+        <v>/Icons/football.svg</v>
       </c>
       <c r="D8" t="str">
         <v>The beautiful game played between two teams of eleven players each.</v>
@@ -524,7 +524,7 @@
         <v>Basketball</v>
       </c>
       <c r="C9" t="str">
-        <v>/icons/basketball.svg</v>
+        <v>/Icons/basketball.svg</v>
       </c>
       <c r="D9" t="str">
         <v>Fast-paced team sport played with a ball and hoop, requiring coordination and teamwork.</v>
@@ -538,7 +538,7 @@
         <v>Lemon Spoon Race</v>
       </c>
       <c r="C10" t="str">
-        <v>/icons/lemon-spoon.svg</v>
+        <v>/Icons/lemon-spoon.svg</v>
       </c>
       <c r="D10" t="str">
         <v>Fun relay race where participants balance a lemon on a spoon while running.</v>

</xml_diff>